<commit_message>
Update step-by-step guide and settings workbook
</commit_message>
<xml_diff>
--- a/settings_configuration.xlsx
+++ b/settings_configuration.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\COBRA\GITHUB\GO to GITHUB\ROC_tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9352B4EC-DA64-4EC6-A85F-9F27979986ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{532904B7-4983-45BE-8AB2-986C8A22B2EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12690" yWindow="0" windowWidth="13020" windowHeight="20985" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3045" yWindow="1335" windowWidth="35355" windowHeight="19545" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -393,12 +393,6 @@
     <t>Year</t>
   </si>
   <si>
-    <t>biotic.xlsx</t>
-  </si>
-  <si>
-    <t>abiotic.xlsx</t>
-  </si>
-  <si>
     <t>abio_infile</t>
   </si>
   <si>
@@ -436,6 +430,12 @@
   </si>
   <si>
     <t>Minimum deseasoned monthly observations required for ABIO trend estimation.</t>
+  </si>
+  <si>
+    <t>abiotic_data_example.xlsx</t>
+  </si>
+  <si>
+    <t>biotic_data_example.xlsx</t>
   </si>
 </sst>
 </file>
@@ -890,7 +890,7 @@
         <v>37</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>38</v>
@@ -898,13 +898,13 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -920,7 +920,7 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B8" s="7" t="b">
         <v>1</v>
@@ -1030,7 +1030,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>56</v>
@@ -1073,7 +1073,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>58</v>
@@ -1084,7 +1084,7 @@
         <v>59</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>60</v>
@@ -1209,7 +1209,7 @@
         <v>0.25</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1220,7 +1220,7 @@
         <v>114</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="28.5">
@@ -1283,7 +1283,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="6" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>81</v>
@@ -1306,7 +1306,7 @@
         <v>50</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -1357,7 +1357,7 @@
         <v>87</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="28.5">
@@ -1776,10 +1776,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="28.5">
@@ -1790,7 +1790,7 @@
         <v>24</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="28.5">

</xml_diff>